<commit_message>
Wire B: AAPL test forecast — Scenarios Consensus C5=0.03, C6=0.025, C7=0.03
</commit_message>
<xml_diff>
--- a/MODEL_TEMPLATE.xlsx
+++ b/MODEL_TEMPLATE.xlsx
@@ -5258,7 +5258,7 @@
         <v>-0.015</v>
       </c>
       <c r="C5" s="89" t="n">
-        <v>0.005</v>
+        <v>0.03</v>
       </c>
       <c r="D5" s="89" t="n">
         <v>0.025</v>
@@ -5277,7 +5277,7 @@
         <v>-0.01</v>
       </c>
       <c r="C6" s="89" t="n">
-        <v>0.01</v>
+        <v>0.025</v>
       </c>
       <c r="D6" s="89" t="n">
         <v>0.03</v>
@@ -5296,7 +5296,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="89" t="n">
-        <v>0.019</v>
+        <v>0.03</v>
       </c>
       <c r="D7" s="89" t="n">
         <v>0.03</v>

</xml_diff>

<commit_message>
Increment 1: depreciation tax penalty (tax on reported EBIT)
Anchor (Econ Statements r52) + forecast (r16) now charge unlevered cash tax
on reported/historical-cost EBIT rather than economic OI. Introduces the
t*shortfall depreciation penalty (non-neutrality #1). Ties preserved across
all 5 tickers (AAPL/T/HD/POOL/AZO), incl. AZO negative-equity + POOL short-history.

WIP / DO NOT MERGE: HD shows +5.1% because reported D&A (4176) ~2x PP&E-based
economic dep (2148) — likely lease/intangible amortization not in gross PP&E.
Resolve the D&A-composition (apples-to-apples) question before merge. Golden
AAPL fixture needs updating (AAPL +0.6%).
</commit_message>
<xml_diff>
--- a/MODEL_TEMPLATE.xlsx
+++ b/MODEL_TEMPLATE.xlsx
@@ -40312,75 +40312,75 @@
         </is>
       </c>
       <c r="B52" s="101">
-        <f>B51*(1-B24)</f>
+        <f>(B51-B24*B20*B6)</f>
         <v/>
       </c>
       <c r="C52" s="101">
-        <f>C51*(1-C24)</f>
+        <f>(C51-C24*C20*C6)</f>
         <v/>
       </c>
       <c r="D52" s="101">
-        <f>D51*(1-D24)</f>
+        <f>(D51-D24*D20*D6)</f>
         <v/>
       </c>
       <c r="E52" s="101">
-        <f>E51*(1-E24)</f>
+        <f>(E51-E24*E20*E6)</f>
         <v/>
       </c>
       <c r="F52" s="101">
-        <f>F51*(1-F24)</f>
+        <f>(F51-F24*F20*F6)</f>
         <v/>
       </c>
       <c r="G52" s="101">
-        <f>G51*(1-G24)</f>
+        <f>(G51-G24*G20*G6)</f>
         <v/>
       </c>
       <c r="H52" s="101">
-        <f>H51*(1-H24)</f>
+        <f>(H51-H24*H20*H6)</f>
         <v/>
       </c>
       <c r="I52" s="101">
-        <f>I51*(1-I24)</f>
+        <f>(I51-I24*I20*I6)</f>
         <v/>
       </c>
       <c r="J52" s="101">
-        <f>J51*(1-J24)</f>
+        <f>(J51-J24*J20*J6)</f>
         <v/>
       </c>
       <c r="K52" s="101">
-        <f>K51*(1-K24)</f>
+        <f>(K51-K24*K20*K6)</f>
         <v/>
       </c>
       <c r="L52" s="101">
-        <f>L51*(1-L24)</f>
+        <f>(L51-L24*L20*L6)</f>
         <v/>
       </c>
       <c r="M52" s="101">
-        <f>M51*(1-M24)</f>
+        <f>(M51-M24*M20*M6)</f>
         <v/>
       </c>
       <c r="N52" s="101">
-        <f>N51*(1-N24)</f>
+        <f>(N51-N24*N20*N6)</f>
         <v/>
       </c>
       <c r="O52" s="101">
-        <f>O51*(1-O24)</f>
+        <f>(O51-O24*O20*O6)</f>
         <v/>
       </c>
       <c r="P52" s="101">
-        <f>P51*(1-P24)</f>
+        <f>(P51-P24*P20*P6)</f>
         <v/>
       </c>
       <c r="Q52" s="101">
-        <f>Q51*(1-Q24)</f>
+        <f>(Q51-Q24*Q20*Q6)</f>
         <v/>
       </c>
       <c r="R52" s="101">
-        <f>R51*(1-R24)</f>
+        <f>(R51-R24*R20*R6)</f>
         <v/>
       </c>
       <c r="S52" s="101">
-        <f>S51*(1-S24)</f>
+        <f>(S51-S24*S20*S6)</f>
         <v/>
       </c>
     </row>
@@ -45153,123 +45153,123 @@
         <v/>
       </c>
       <c r="G16" s="101">
-        <f>IF(G4&lt;=cfg_N,G15*(1-G17),G60*F24)</f>
+        <f>IF(G4&lt;=cfg_N,(G15*(1-G17)-G17*G13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),G60*F24)</f>
         <v/>
       </c>
       <c r="H16" s="101">
-        <f>IF(H4&lt;=cfg_N,H15*(1-H17),H60*G24)</f>
+        <f>IF(H4&lt;=cfg_N,(H15*(1-H17)-H17*H13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),H60*G24)</f>
         <v/>
       </c>
       <c r="I16" s="101">
-        <f>IF(I4&lt;=cfg_N,I15*(1-I17),I60*H24)</f>
+        <f>IF(I4&lt;=cfg_N,(I15*(1-I17)-I17*I13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),I60*H24)</f>
         <v/>
       </c>
       <c r="J16" s="101">
-        <f>IF(J4&lt;=cfg_N,J15*(1-J17),J60*I24)</f>
+        <f>IF(J4&lt;=cfg_N,(J15*(1-J17)-J17*J13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),J60*I24)</f>
         <v/>
       </c>
       <c r="K16" s="101">
-        <f>IF(K4&lt;=cfg_N,K15*(1-K17),K60*J24)</f>
+        <f>IF(K4&lt;=cfg_N,(K15*(1-K17)-K17*K13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),K60*J24)</f>
         <v/>
       </c>
       <c r="L16" s="101">
-        <f>IF(L4&lt;=cfg_N,L15*(1-L17),L60*K24)</f>
+        <f>IF(L4&lt;=cfg_N,(L15*(1-L17)-L17*L13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),L60*K24)</f>
         <v/>
       </c>
       <c r="M16" s="101">
-        <f>IF(M4&lt;=cfg_N,M15*(1-M17),M60*L24)</f>
+        <f>IF(M4&lt;=cfg_N,(M15*(1-M17)-M17*M13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),M60*L24)</f>
         <v/>
       </c>
       <c r="N16" s="101">
-        <f>IF(N4&lt;=cfg_N,N15*(1-N17),N60*M24)</f>
+        <f>IF(N4&lt;=cfg_N,(N15*(1-N17)-N17*N13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),N60*M24)</f>
         <v/>
       </c>
       <c r="O16" s="101">
-        <f>IF(O4&lt;=cfg_N,O15*(1-O17),O60*N24)</f>
+        <f>IF(O4&lt;=cfg_N,(O15*(1-O17)-O17*O13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),O60*N24)</f>
         <v/>
       </c>
       <c r="P16" s="101">
-        <f>IF(P4&lt;=cfg_N,P15*(1-P17),P60*O24)</f>
+        <f>IF(P4&lt;=cfg_N,(P15*(1-P17)-P17*P13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),P60*O24)</f>
         <v/>
       </c>
       <c r="Q16" s="101">
-        <f>IF(Q4&lt;=cfg_N,Q15*(1-Q17),Q60*P24)</f>
+        <f>IF(Q4&lt;=cfg_N,(Q15*(1-Q17)-Q17*Q13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Q60*P24)</f>
         <v/>
       </c>
       <c r="R16" s="101">
-        <f>IF(R4&lt;=cfg_N,R15*(1-R17),R60*Q24)</f>
+        <f>IF(R4&lt;=cfg_N,(R15*(1-R17)-R17*R13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),R60*Q24)</f>
         <v/>
       </c>
       <c r="S16" s="101">
-        <f>IF(S4&lt;=cfg_N,S15*(1-S17),S60*R24)</f>
+        <f>IF(S4&lt;=cfg_N,(S15*(1-S17)-S17*S13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),S60*R24)</f>
         <v/>
       </c>
       <c r="T16" s="86">
-        <f>IF(T4&lt;=cfg_N,T15*(1-T17),T60*S24)</f>
+        <f>IF(T4&lt;=cfg_N,(T15*(1-T17)-T17*T13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),T60*S24)</f>
         <v/>
       </c>
       <c r="U16" s="86">
-        <f>IF(U4&lt;=cfg_N,U15*(1-U17),U60*T24)</f>
+        <f>IF(U4&lt;=cfg_N,(U15*(1-U17)-U17*U13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),U60*T24)</f>
         <v/>
       </c>
       <c r="V16" s="86">
-        <f>IF(V4&lt;=cfg_N,V15*(1-V17),V60*U24)</f>
+        <f>IF(V4&lt;=cfg_N,(V15*(1-V17)-V17*V13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),V60*U24)</f>
         <v/>
       </c>
       <c r="W16" s="86">
-        <f>IF(W4&lt;=cfg_N,W15*(1-W17),W60*V24)</f>
+        <f>IF(W4&lt;=cfg_N,(W15*(1-W17)-W17*W13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),W60*V24)</f>
         <v/>
       </c>
       <c r="X16" s="86">
-        <f>IF(X4&lt;=cfg_N,X15*(1-X17),X60*W24)</f>
+        <f>IF(X4&lt;=cfg_N,(X15*(1-X17)-X17*X13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),X60*W24)</f>
         <v/>
       </c>
       <c r="Y16" s="86">
-        <f>IF(Y4&lt;=cfg_N,Y15*(1-Y17),Y60*X24)</f>
+        <f>IF(Y4&lt;=cfg_N,(Y15*(1-Y17)-Y17*Y13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Y60*X24)</f>
         <v/>
       </c>
       <c r="Z16" s="86">
-        <f>IF(Z4&lt;=cfg_N,Z15*(1-Z17),Z60*Y24)</f>
+        <f>IF(Z4&lt;=cfg_N,(Z15*(1-Z17)-Z17*Z13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Z60*Y24)</f>
         <v/>
       </c>
       <c r="AA16" s="86">
-        <f>IF(AA4&lt;=cfg_N,AA15*(1-AA17),AA60*Z24)</f>
+        <f>IF(AA4&lt;=cfg_N,(AA15*(1-AA17)-AA17*AA13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AA60*Z24)</f>
         <v/>
       </c>
       <c r="AB16" s="86">
-        <f>IF(AB4&lt;=cfg_N,AB15*(1-AB17),AB60*AA24)</f>
+        <f>IF(AB4&lt;=cfg_N,(AB15*(1-AB17)-AB17*AB13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AB60*AA24)</f>
         <v/>
       </c>
       <c r="AC16" s="86">
-        <f>IF(AC4&lt;=cfg_N,AC15*(1-AC17),AC60*AB24)</f>
+        <f>IF(AC4&lt;=cfg_N,(AC15*(1-AC17)-AC17*AC13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AC60*AB24)</f>
         <v/>
       </c>
       <c r="AD16" s="86">
-        <f>IF(AD4&lt;=cfg_N,AD15*(1-AD17),AD60*AC24)</f>
+        <f>IF(AD4&lt;=cfg_N,(AD15*(1-AD17)-AD17*AD13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AD60*AC24)</f>
         <v/>
       </c>
       <c r="AE16" s="86">
-        <f>IF(AE4&lt;=cfg_N,AE15*(1-AE17),AE60*AD24)</f>
+        <f>IF(AE4&lt;=cfg_N,(AE15*(1-AE17)-AE17*AE13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AE60*AD24)</f>
         <v/>
       </c>
       <c r="AF16" s="86">
-        <f>IF(AF4&lt;=cfg_N,AF15*(1-AF17),AF60*AE24)</f>
+        <f>IF(AF4&lt;=cfg_N,(AF15*(1-AF17)-AF17*AF13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AF60*AE24)</f>
         <v/>
       </c>
       <c r="AG16" s="86">
-        <f>IF(AG4&lt;=cfg_N,AG15*(1-AG17),AG60*AF24)</f>
+        <f>IF(AG4&lt;=cfg_N,(AG15*(1-AG17)-AG17*AG13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AG60*AF24)</f>
         <v/>
       </c>
       <c r="AH16" s="86">
-        <f>IF(AH4&lt;=cfg_N,AH15*(1-AH17),AH60*AG24)</f>
+        <f>IF(AH4&lt;=cfg_N,(AH15*(1-AH17)-AH17*AH13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AH60*AG24)</f>
         <v/>
       </c>
       <c r="AI16" s="86">
-        <f>IF(AI4&lt;=cfg_N,AI15*(1-AI17),AI60*AH24)</f>
+        <f>IF(AI4&lt;=cfg_N,(AI15*(1-AI17)-AI17*AI13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AI60*AH24)</f>
         <v/>
       </c>
       <c r="AJ16" s="86">
-        <f>IF(AJ4&lt;=cfg_N,AJ15*(1-AJ17),AJ60*AI24)</f>
+        <f>IF(AJ4&lt;=cfg_N,(AJ15*(1-AJ17)-AJ17*AJ13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AJ60*AI24)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Increment 1 (corrected): PP&E-scoped depreciation penalty, wedge-safe
Fixes two errors in the prior WIP commit:
1. Shortfall now pairs current-cost vs historical-cost depreciation of the SAME
   live vintages (SUMPRODUCT of nominal capex x live-flag, over Cap Engine's
   vintage table), not economic dep vs reported TOTAL D&A. Removes the spurious
   HD +5% (lease/intangible amort is no longer miscounted).
2. Re-points Forecast!F15 (period-0 pre-tax EBIT) to the true economic OI pretax
   ('Econ Statements'!S51) instead of anchor_oi_at0/(1-t). The penalty is an extra
   (non-flat) tax; the old gross-up leaked it into the opex-wedge gate (tripped T).

Result: all 5 tickers tie to machine precision, opex-wedge stays 0, and every name
shows a sensible depreciation PENALTY scaling with capital intensity/asset age:
AAPL -0.16%, POOL -0.23%, HD -0.26%, AZO -0.69%, T -1.81%.

TODO before merge: refresh golden AAPL fixture (AAPL moved -0.16%).
</commit_message>
<xml_diff>
--- a/MODEL_TEMPLATE.xlsx
+++ b/MODEL_TEMPLATE.xlsx
@@ -40312,75 +40312,75 @@
         </is>
       </c>
       <c r="B52" s="101">
-        <f>(B51-B24*B20*B6)</f>
+        <f>(B51*(1-B24)-B24*B50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="C52" s="101">
-        <f>(C51-C24*C20*C6)</f>
+        <f>(C51*(1-C24)-C24*C50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="D52" s="101">
-        <f>(D51-D24*D20*D6)</f>
+        <f>(D51*(1-D24)-D24*D50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="E52" s="101">
-        <f>(E51-E24*E20*E6)</f>
+        <f>(E51*(1-E24)-E24*E50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="F52" s="101">
-        <f>(F51-F24*F20*F6)</f>
+        <f>(F51*(1-F24)-F24*F50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="G52" s="101">
-        <f>(G51-G24*G20*G6)</f>
+        <f>(G51*(1-G24)-G24*G50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="H52" s="101">
-        <f>(H51-H24*H20*H6)</f>
+        <f>(H51*(1-H24)-H24*H50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="I52" s="101">
-        <f>(I51-I24*I20*I6)</f>
+        <f>(I51*(1-I24)-I24*I50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="J52" s="101">
-        <f>(J51-J24*J20*J6)</f>
+        <f>(J51*(1-J24)-J24*J50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="K52" s="101">
-        <f>(K51-K24*K20*K6)</f>
+        <f>(K51*(1-K24)-K24*K50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="L52" s="101">
-        <f>(L51-L24*L20*L6)</f>
+        <f>(L51*(1-L24)-L24*L50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="M52" s="101">
-        <f>(M51-M24*M20*M6)</f>
+        <f>(M51*(1-M24)-M24*M50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="N52" s="101">
-        <f>(N51-N24*N20*N6)</f>
+        <f>(N51*(1-N24)-N24*N50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="O52" s="101">
-        <f>(O51-O24*O20*O6)</f>
+        <f>(O51*(1-O24)-O24*O50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="P52" s="101">
-        <f>(P51-P24*P20*P6)</f>
+        <f>(P51*(1-P24)-P24*P50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="Q52" s="101">
-        <f>(Q51-Q24*Q20*Q6)</f>
+        <f>(Q51*(1-Q24)-Q24*Q50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="R52" s="101">
-        <f>(R51-R24*R20*R6)</f>
+        <f>(R51*(1-R24)-R24*R50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="S52" s="101">
-        <f>(S51-S24*S20*S6)</f>
+        <f>(S51*(1-S24)-S24*S50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
     </row>
@@ -45006,7 +45006,7 @@
         <v/>
       </c>
       <c r="F15" s="101">
-        <f>anchor_oi_at0/(1-$F$17)</f>
+        <f>'Econ Statements'!$S$51</f>
         <v/>
       </c>
       <c r="G15" s="101">
@@ -45153,123 +45153,123 @@
         <v/>
       </c>
       <c r="G16" s="101">
-        <f>IF(G4&lt;=cfg_N,(G15*(1-G17)-G17*G13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),G60*F24)</f>
+        <f>IF(G4&lt;=cfg_N,(G15*(1-G17)-G17*G13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),G60*F24)</f>
         <v/>
       </c>
       <c r="H16" s="101">
-        <f>IF(H4&lt;=cfg_N,(H15*(1-H17)-H17*H13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),H60*G24)</f>
+        <f>IF(H4&lt;=cfg_N,(H15*(1-H17)-H17*H13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),H60*G24)</f>
         <v/>
       </c>
       <c r="I16" s="101">
-        <f>IF(I4&lt;=cfg_N,(I15*(1-I17)-I17*I13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),I60*H24)</f>
+        <f>IF(I4&lt;=cfg_N,(I15*(1-I17)-I17*I13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),I60*H24)</f>
         <v/>
       </c>
       <c r="J16" s="101">
-        <f>IF(J4&lt;=cfg_N,(J15*(1-J17)-J17*J13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),J60*I24)</f>
+        <f>IF(J4&lt;=cfg_N,(J15*(1-J17)-J17*J13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),J60*I24)</f>
         <v/>
       </c>
       <c r="K16" s="101">
-        <f>IF(K4&lt;=cfg_N,(K15*(1-K17)-K17*K13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),K60*J24)</f>
+        <f>IF(K4&lt;=cfg_N,(K15*(1-K17)-K17*K13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),K60*J24)</f>
         <v/>
       </c>
       <c r="L16" s="101">
-        <f>IF(L4&lt;=cfg_N,(L15*(1-L17)-L17*L13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),L60*K24)</f>
+        <f>IF(L4&lt;=cfg_N,(L15*(1-L17)-L17*L13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),L60*K24)</f>
         <v/>
       </c>
       <c r="M16" s="101">
-        <f>IF(M4&lt;=cfg_N,(M15*(1-M17)-M17*M13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),M60*L24)</f>
+        <f>IF(M4&lt;=cfg_N,(M15*(1-M17)-M17*M13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),M60*L24)</f>
         <v/>
       </c>
       <c r="N16" s="101">
-        <f>IF(N4&lt;=cfg_N,(N15*(1-N17)-N17*N13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),N60*M24)</f>
+        <f>IF(N4&lt;=cfg_N,(N15*(1-N17)-N17*N13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),N60*M24)</f>
         <v/>
       </c>
       <c r="O16" s="101">
-        <f>IF(O4&lt;=cfg_N,(O15*(1-O17)-O17*O13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),O60*N24)</f>
+        <f>IF(O4&lt;=cfg_N,(O15*(1-O17)-O17*O13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),O60*N24)</f>
         <v/>
       </c>
       <c r="P16" s="101">
-        <f>IF(P4&lt;=cfg_N,(P15*(1-P17)-P17*P13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),P60*O24)</f>
+        <f>IF(P4&lt;=cfg_N,(P15*(1-P17)-P17*P13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),P60*O24)</f>
         <v/>
       </c>
       <c r="Q16" s="101">
-        <f>IF(Q4&lt;=cfg_N,(Q15*(1-Q17)-Q17*Q13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Q60*P24)</f>
+        <f>IF(Q4&lt;=cfg_N,(Q15*(1-Q17)-Q17*Q13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Q60*P24)</f>
         <v/>
       </c>
       <c r="R16" s="101">
-        <f>IF(R4&lt;=cfg_N,(R15*(1-R17)-R17*R13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),R60*Q24)</f>
+        <f>IF(R4&lt;=cfg_N,(R15*(1-R17)-R17*R13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),R60*Q24)</f>
         <v/>
       </c>
       <c r="S16" s="101">
-        <f>IF(S4&lt;=cfg_N,(S15*(1-S17)-S17*S13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),S60*R24)</f>
+        <f>IF(S4&lt;=cfg_N,(S15*(1-S17)-S17*S13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),S60*R24)</f>
         <v/>
       </c>
       <c r="T16" s="86">
-        <f>IF(T4&lt;=cfg_N,(T15*(1-T17)-T17*T13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),T60*S24)</f>
+        <f>IF(T4&lt;=cfg_N,(T15*(1-T17)-T17*T13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),T60*S24)</f>
         <v/>
       </c>
       <c r="U16" s="86">
-        <f>IF(U4&lt;=cfg_N,(U15*(1-U17)-U17*U13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),U60*T24)</f>
+        <f>IF(U4&lt;=cfg_N,(U15*(1-U17)-U17*U13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),U60*T24)</f>
         <v/>
       </c>
       <c r="V16" s="86">
-        <f>IF(V4&lt;=cfg_N,(V15*(1-V17)-V17*V13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),V60*U24)</f>
+        <f>IF(V4&lt;=cfg_N,(V15*(1-V17)-V17*V13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),V60*U24)</f>
         <v/>
       </c>
       <c r="W16" s="86">
-        <f>IF(W4&lt;=cfg_N,(W15*(1-W17)-W17*W13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),W60*V24)</f>
+        <f>IF(W4&lt;=cfg_N,(W15*(1-W17)-W17*W13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),W60*V24)</f>
         <v/>
       </c>
       <c r="X16" s="86">
-        <f>IF(X4&lt;=cfg_N,(X15*(1-X17)-X17*X13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),X60*W24)</f>
+        <f>IF(X4&lt;=cfg_N,(X15*(1-X17)-X17*X13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),X60*W24)</f>
         <v/>
       </c>
       <c r="Y16" s="86">
-        <f>IF(Y4&lt;=cfg_N,(Y15*(1-Y17)-Y17*Y13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Y60*X24)</f>
+        <f>IF(Y4&lt;=cfg_N,(Y15*(1-Y17)-Y17*Y13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Y60*X24)</f>
         <v/>
       </c>
       <c r="Z16" s="86">
-        <f>IF(Z4&lt;=cfg_N,(Z15*(1-Z17)-Z17*Z13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),Z60*Y24)</f>
+        <f>IF(Z4&lt;=cfg_N,(Z15*(1-Z17)-Z17*Z13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Z60*Y24)</f>
         <v/>
       </c>
       <c r="AA16" s="86">
-        <f>IF(AA4&lt;=cfg_N,(AA15*(1-AA17)-AA17*AA13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AA60*Z24)</f>
+        <f>IF(AA4&lt;=cfg_N,(AA15*(1-AA17)-AA17*AA13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AA60*Z24)</f>
         <v/>
       </c>
       <c r="AB16" s="86">
-        <f>IF(AB4&lt;=cfg_N,(AB15*(1-AB17)-AB17*AB13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AB60*AA24)</f>
+        <f>IF(AB4&lt;=cfg_N,(AB15*(1-AB17)-AB17*AB13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AB60*AA24)</f>
         <v/>
       </c>
       <c r="AC16" s="86">
-        <f>IF(AC4&lt;=cfg_N,(AC15*(1-AC17)-AC17*AC13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AC60*AB24)</f>
+        <f>IF(AC4&lt;=cfg_N,(AC15*(1-AC17)-AC17*AC13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AC60*AB24)</f>
         <v/>
       </c>
       <c r="AD16" s="86">
-        <f>IF(AD4&lt;=cfg_N,(AD15*(1-AD17)-AD17*AD13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AD60*AC24)</f>
+        <f>IF(AD4&lt;=cfg_N,(AD15*(1-AD17)-AD17*AD13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AD60*AC24)</f>
         <v/>
       </c>
       <c r="AE16" s="86">
-        <f>IF(AE4&lt;=cfg_N,(AE15*(1-AE17)-AE17*AE13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AE60*AD24)</f>
+        <f>IF(AE4&lt;=cfg_N,(AE15*(1-AE17)-AE17*AE13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AE60*AD24)</f>
         <v/>
       </c>
       <c r="AF16" s="86">
-        <f>IF(AF4&lt;=cfg_N,(AF15*(1-AF17)-AF17*AF13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AF60*AE24)</f>
+        <f>IF(AF4&lt;=cfg_N,(AF15*(1-AF17)-AF17*AF13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AF60*AE24)</f>
         <v/>
       </c>
       <c r="AG16" s="86">
-        <f>IF(AG4&lt;=cfg_N,(AG15*(1-AG17)-AG17*AG13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AG60*AF24)</f>
+        <f>IF(AG4&lt;=cfg_N,(AG15*(1-AG17)-AG17*AG13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AG60*AF24)</f>
         <v/>
       </c>
       <c r="AH16" s="86">
-        <f>IF(AH4&lt;=cfg_N,(AH15*(1-AH17)-AH17*AH13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AH60*AG24)</f>
+        <f>IF(AH4&lt;=cfg_N,(AH15*(1-AH17)-AH17*AH13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AH60*AG24)</f>
         <v/>
       </c>
       <c r="AI16" s="86">
-        <f>IF(AI4&lt;=cfg_N,(AI15*(1-AI17)-AI17*AI13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AI60*AH24)</f>
+        <f>IF(AI4&lt;=cfg_N,(AI15*(1-AI17)-AI17*AI13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AI60*AH24)</f>
         <v/>
       </c>
       <c r="AJ16" s="86">
-        <f>IF(AJ4&lt;=cfg_N,(AJ15*(1-AJ17)-AJ17*AJ13*(1-('Econ Statements'!$S$21*'Econ Statements'!$S$6)/'Econ Statements'!$S$50)),AJ60*AI24)</f>
+        <f>IF(AJ4&lt;=cfg_N,(AJ15*(1-AJ17)-AJ17*AJ13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AJ60*AI24)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Increment 1: PP&E-scoped depreciation tax penalty (inflation non-neutrality #1)
Charge unlevered cash tax on historical-cost (reported) PP&E depreciation rather
than current-cost economic depreciation, capturing the t*shortfall penalty the
real-terms frame previously assumed away. Shortfall pairs current-cost vs
historical-cost depreciation of the SAME live vintages (Cap Engine vintage table);
Forecast!F15 re-pointed to true pre-tax OI so the extra tax stays in the tax line
and does not perturb the opex-wedge gate.

Ties preserved to machine precision on all 5 tickers + the full regression grid.
Per-name effect (equity): AAPL -0.16%, POOL -0.23%, HD -0.26%, AZO -0.69%, T -1.81%
— scales with capital intensity / asset age, as predicted.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UFSrGmX9ywdAsZo9EWtx68
</commit_message>
<xml_diff>
--- a/MODEL_TEMPLATE.xlsx
+++ b/MODEL_TEMPLATE.xlsx
@@ -40312,75 +40312,75 @@
         </is>
       </c>
       <c r="B52" s="101">
-        <f>B51*(1-B24)</f>
+        <f>(B51*(1-B24)-B24*B50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="C52" s="101">
-        <f>C51*(1-C24)</f>
+        <f>(C51*(1-C24)-C24*C50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="D52" s="101">
-        <f>D51*(1-D24)</f>
+        <f>(D51*(1-D24)-D24*D50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="E52" s="101">
-        <f>E51*(1-E24)</f>
+        <f>(E51*(1-E24)-E24*E50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="F52" s="101">
-        <f>F51*(1-F24)</f>
+        <f>(F51*(1-F24)-F24*F50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="G52" s="101">
-        <f>G51*(1-G24)</f>
+        <f>(G51*(1-G24)-G24*G50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="H52" s="101">
-        <f>H51*(1-H24)</f>
+        <f>(H51*(1-H24)-H24*H50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="I52" s="101">
-        <f>I51*(1-I24)</f>
+        <f>(I51*(1-I24)-I24*I50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="J52" s="101">
-        <f>J51*(1-J24)</f>
+        <f>(J51*(1-J24)-J24*J50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="K52" s="101">
-        <f>K51*(1-K24)</f>
+        <f>(K51*(1-K24)-K24*K50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="L52" s="101">
-        <f>L51*(1-L24)</f>
+        <f>(L51*(1-L24)-L24*L50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="M52" s="101">
-        <f>M51*(1-M24)</f>
+        <f>(M51*(1-M24)-M24*M50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="N52" s="101">
-        <f>N51*(1-N24)</f>
+        <f>(N51*(1-N24)-N24*N50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="O52" s="101">
-        <f>O51*(1-O24)</f>
+        <f>(O51*(1-O24)-O24*O50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="P52" s="101">
-        <f>P51*(1-P24)</f>
+        <f>(P51*(1-P24)-P24*P50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="Q52" s="101">
-        <f>Q51*(1-Q24)</f>
+        <f>(Q51*(1-Q24)-Q24*Q50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="R52" s="101">
-        <f>R51*(1-R24)</f>
+        <f>(R51*(1-R24)-R24*R50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
       <c r="S52" s="101">
-        <f>S51*(1-S24)</f>
+        <f>(S51*(1-S24)-S24*S50*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46))</f>
         <v/>
       </c>
     </row>
@@ -45006,7 +45006,7 @@
         <v/>
       </c>
       <c r="F15" s="101">
-        <f>anchor_oi_at0/(1-$F$17)</f>
+        <f>'Econ Statements'!$S$51</f>
         <v/>
       </c>
       <c r="G15" s="101">
@@ -45153,123 +45153,123 @@
         <v/>
       </c>
       <c r="G16" s="101">
-        <f>IF(G4&lt;=cfg_N,G15*(1-G17),G60*F24)</f>
+        <f>IF(G4&lt;=cfg_N,(G15*(1-G17)-G17*G13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),G60*F24)</f>
         <v/>
       </c>
       <c r="H16" s="101">
-        <f>IF(H4&lt;=cfg_N,H15*(1-H17),H60*G24)</f>
+        <f>IF(H4&lt;=cfg_N,(H15*(1-H17)-H17*H13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),H60*G24)</f>
         <v/>
       </c>
       <c r="I16" s="101">
-        <f>IF(I4&lt;=cfg_N,I15*(1-I17),I60*H24)</f>
+        <f>IF(I4&lt;=cfg_N,(I15*(1-I17)-I17*I13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),I60*H24)</f>
         <v/>
       </c>
       <c r="J16" s="101">
-        <f>IF(J4&lt;=cfg_N,J15*(1-J17),J60*I24)</f>
+        <f>IF(J4&lt;=cfg_N,(J15*(1-J17)-J17*J13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),J60*I24)</f>
         <v/>
       </c>
       <c r="K16" s="101">
-        <f>IF(K4&lt;=cfg_N,K15*(1-K17),K60*J24)</f>
+        <f>IF(K4&lt;=cfg_N,(K15*(1-K17)-K17*K13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),K60*J24)</f>
         <v/>
       </c>
       <c r="L16" s="101">
-        <f>IF(L4&lt;=cfg_N,L15*(1-L17),L60*K24)</f>
+        <f>IF(L4&lt;=cfg_N,(L15*(1-L17)-L17*L13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),L60*K24)</f>
         <v/>
       </c>
       <c r="M16" s="101">
-        <f>IF(M4&lt;=cfg_N,M15*(1-M17),M60*L24)</f>
+        <f>IF(M4&lt;=cfg_N,(M15*(1-M17)-M17*M13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),M60*L24)</f>
         <v/>
       </c>
       <c r="N16" s="101">
-        <f>IF(N4&lt;=cfg_N,N15*(1-N17),N60*M24)</f>
+        <f>IF(N4&lt;=cfg_N,(N15*(1-N17)-N17*N13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),N60*M24)</f>
         <v/>
       </c>
       <c r="O16" s="101">
-        <f>IF(O4&lt;=cfg_N,O15*(1-O17),O60*N24)</f>
+        <f>IF(O4&lt;=cfg_N,(O15*(1-O17)-O17*O13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),O60*N24)</f>
         <v/>
       </c>
       <c r="P16" s="101">
-        <f>IF(P4&lt;=cfg_N,P15*(1-P17),P60*O24)</f>
+        <f>IF(P4&lt;=cfg_N,(P15*(1-P17)-P17*P13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),P60*O24)</f>
         <v/>
       </c>
       <c r="Q16" s="101">
-        <f>IF(Q4&lt;=cfg_N,Q15*(1-Q17),Q60*P24)</f>
+        <f>IF(Q4&lt;=cfg_N,(Q15*(1-Q17)-Q17*Q13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Q60*P24)</f>
         <v/>
       </c>
       <c r="R16" s="101">
-        <f>IF(R4&lt;=cfg_N,R15*(1-R17),R60*Q24)</f>
+        <f>IF(R4&lt;=cfg_N,(R15*(1-R17)-R17*R13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),R60*Q24)</f>
         <v/>
       </c>
       <c r="S16" s="101">
-        <f>IF(S4&lt;=cfg_N,S15*(1-S17),S60*R24)</f>
+        <f>IF(S4&lt;=cfg_N,(S15*(1-S17)-S17*S13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),S60*R24)</f>
         <v/>
       </c>
       <c r="T16" s="86">
-        <f>IF(T4&lt;=cfg_N,T15*(1-T17),T60*S24)</f>
+        <f>IF(T4&lt;=cfg_N,(T15*(1-T17)-T17*T13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),T60*S24)</f>
         <v/>
       </c>
       <c r="U16" s="86">
-        <f>IF(U4&lt;=cfg_N,U15*(1-U17),U60*T24)</f>
+        <f>IF(U4&lt;=cfg_N,(U15*(1-U17)-U17*U13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),U60*T24)</f>
         <v/>
       </c>
       <c r="V16" s="86">
-        <f>IF(V4&lt;=cfg_N,V15*(1-V17),V60*U24)</f>
+        <f>IF(V4&lt;=cfg_N,(V15*(1-V17)-V17*V13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),V60*U24)</f>
         <v/>
       </c>
       <c r="W16" s="86">
-        <f>IF(W4&lt;=cfg_N,W15*(1-W17),W60*V24)</f>
+        <f>IF(W4&lt;=cfg_N,(W15*(1-W17)-W17*W13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),W60*V24)</f>
         <v/>
       </c>
       <c r="X16" s="86">
-        <f>IF(X4&lt;=cfg_N,X15*(1-X17),X60*W24)</f>
+        <f>IF(X4&lt;=cfg_N,(X15*(1-X17)-X17*X13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),X60*W24)</f>
         <v/>
       </c>
       <c r="Y16" s="86">
-        <f>IF(Y4&lt;=cfg_N,Y15*(1-Y17),Y60*X24)</f>
+        <f>IF(Y4&lt;=cfg_N,(Y15*(1-Y17)-Y17*Y13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Y60*X24)</f>
         <v/>
       </c>
       <c r="Z16" s="86">
-        <f>IF(Z4&lt;=cfg_N,Z15*(1-Z17),Z60*Y24)</f>
+        <f>IF(Z4&lt;=cfg_N,(Z15*(1-Z17)-Z17*Z13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),Z60*Y24)</f>
         <v/>
       </c>
       <c r="AA16" s="86">
-        <f>IF(AA4&lt;=cfg_N,AA15*(1-AA17),AA60*Z24)</f>
+        <f>IF(AA4&lt;=cfg_N,(AA15*(1-AA17)-AA17*AA13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AA60*Z24)</f>
         <v/>
       </c>
       <c r="AB16" s="86">
-        <f>IF(AB4&lt;=cfg_N,AB15*(1-AB17),AB60*AA24)</f>
+        <f>IF(AB4&lt;=cfg_N,(AB15*(1-AB17)-AB17*AB13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AB60*AA24)</f>
         <v/>
       </c>
       <c r="AC16" s="86">
-        <f>IF(AC4&lt;=cfg_N,AC15*(1-AC17),AC60*AB24)</f>
+        <f>IF(AC4&lt;=cfg_N,(AC15*(1-AC17)-AC17*AC13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AC60*AB24)</f>
         <v/>
       </c>
       <c r="AD16" s="86">
-        <f>IF(AD4&lt;=cfg_N,AD15*(1-AD17),AD60*AC24)</f>
+        <f>IF(AD4&lt;=cfg_N,(AD15*(1-AD17)-AD17*AD13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AD60*AC24)</f>
         <v/>
       </c>
       <c r="AE16" s="86">
-        <f>IF(AE4&lt;=cfg_N,AE15*(1-AE17),AE60*AD24)</f>
+        <f>IF(AE4&lt;=cfg_N,(AE15*(1-AE17)-AE17*AE13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AE60*AD24)</f>
         <v/>
       </c>
       <c r="AF16" s="86">
-        <f>IF(AF4&lt;=cfg_N,AF15*(1-AF17),AF60*AE24)</f>
+        <f>IF(AF4&lt;=cfg_N,(AF15*(1-AF17)-AF17*AF13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AF60*AE24)</f>
         <v/>
       </c>
       <c r="AG16" s="86">
-        <f>IF(AG4&lt;=cfg_N,AG15*(1-AG17),AG60*AF24)</f>
+        <f>IF(AG4&lt;=cfg_N,(AG15*(1-AG17)-AG17*AG13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AG60*AF24)</f>
         <v/>
       </c>
       <c r="AH16" s="86">
-        <f>IF(AH4&lt;=cfg_N,AH15*(1-AH17),AH60*AG24)</f>
+        <f>IF(AH4&lt;=cfg_N,(AH15*(1-AH17)-AH17*AH13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AH60*AG24)</f>
         <v/>
       </c>
       <c r="AI16" s="86">
-        <f>IF(AI4&lt;=cfg_N,AI15*(1-AI17),AI60*AH24)</f>
+        <f>IF(AI4&lt;=cfg_N,(AI15*(1-AI17)-AI17*AI13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AI60*AH24)</f>
         <v/>
       </c>
       <c r="AJ16" s="86">
-        <f>IF(AJ4&lt;=cfg_N,AJ15*(1-AJ17),AJ60*AI24)</f>
+        <f>IF(AJ4&lt;=cfg_N,(AJ15*(1-AJ17)-AJ17*AJ13*(1-SUMPRODUCT('Cap Engine'!$B$7:$B$43,'Cap Engine'!$F$7:$F$43)/'Cap Engine'!$B$46)),AJ60*AI24)</f>
         <v/>
       </c>
     </row>

</xml_diff>